<commit_message>
test: use English anonymized fixtures
</commit_message>
<xml_diff>
--- a/test/fixtures/xlsx/01_simple.xlsx
+++ b/test/fixtures/xlsx/01_simple.xlsx
@@ -5,6 +5,26 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample User A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample User B</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>